<commit_message>
update source output files
</commit_message>
<xml_diff>
--- a/CPRD Raw Analysis/Results/Output_costs_Raw-Adjusted.xlsx
+++ b/CPRD Raw Analysis/Results/Output_costs_Raw-Adjusted.xlsx
@@ -414,37 +414,37 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>54617.7</v>
+        <v>1086.33</v>
       </c>
       <c r="B2">
-        <v>1.27</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>10265367.94</v>
+        <v>14096</v>
       </c>
       <c r="D2">
-        <v>173110.34</v>
+        <v>930.0599999999999</v>
       </c>
       <c r="E2">
-        <v>16722.87</v>
+        <v>848.37</v>
       </c>
       <c r="F2">
-        <v>4914.81</v>
+        <v>464.28</v>
       </c>
       <c r="G2">
-        <v>48977.22</v>
+        <v>1428</v>
       </c>
       <c r="H2">
-        <v>15040</v>
+        <v>15088</v>
       </c>
       <c r="I2">
-        <v>1411.559181472828</v>
+        <v>7.571730172132114</v>
       </c>
       <c r="J2">
-        <v>51850.87216348648</v>
+        <v>1071.488490893558</v>
       </c>
       <c r="K2">
-        <v>57384.52783651352</v>
+        <v>1101.171509106442</v>
       </c>
     </row>
   </sheetData>
@@ -516,37 +516,37 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1412.07</v>
+        <v>1098.93</v>
       </c>
       <c r="B2">
-        <v>0.95</v>
+        <v>12</v>
       </c>
       <c r="C2">
-        <v>19934</v>
+        <v>14096</v>
       </c>
       <c r="D2">
-        <v>1280.43</v>
+        <v>928.01</v>
       </c>
       <c r="E2">
-        <v>1081.8</v>
+        <v>862.14</v>
       </c>
       <c r="F2">
-        <v>588</v>
+        <v>482.9</v>
       </c>
       <c r="G2">
-        <v>1841.12</v>
+        <v>1436.37</v>
       </c>
       <c r="H2">
-        <v>14934</v>
+        <v>14915</v>
       </c>
       <c r="I2">
-        <v>10.47774361921209</v>
+        <v>7.598730243541569</v>
       </c>
       <c r="J2">
-        <v>1391.532335229701</v>
+        <v>1084.035553618287</v>
       </c>
       <c r="K2">
-        <v>1432.607664770299</v>
+        <v>1113.824446381713</v>
       </c>
     </row>
   </sheetData>

</xml_diff>